<commit_message>
county data rev & mapping
</commit_message>
<xml_diff>
--- a/data/_countydata.xlsx
+++ b/data/_countydata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27616"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27723"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olekw\Desktop\Studia\MAG  - WNE - Praca magisterska\___towards_final\master_thesis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olekw\Desktop\Studia\MAG  - WNE - Praca magisterska\_____final_remarks\master_thesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44CB69D-8F21-4C46-AD6B-E5B05D120EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38421AE-A39A-4344-8415-24F33AE54D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,132 +41,6 @@
     <t>MAZOWIECKIE</t>
   </si>
   <si>
-    <t>Powiat biaĹ‚obrzeski</t>
-  </si>
-  <si>
-    <t>Powiat ciechanowski</t>
-  </si>
-  <si>
-    <t>Powiat garwoliĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat gostyniĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat grodziski</t>
-  </si>
-  <si>
-    <t>Powiat grĂłjecki</t>
-  </si>
-  <si>
-    <t>Powiat kozienicki</t>
-  </si>
-  <si>
-    <t>Powiat legionowski</t>
-  </si>
-  <si>
-    <t>Powiat lipski</t>
-  </si>
-  <si>
-    <t>Powiat Ĺ‚osicki</t>
-  </si>
-  <si>
-    <t>Powiat makowski</t>
-  </si>
-  <si>
-    <t>Powiat miĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat mĹ‚awski</t>
-  </si>
-  <si>
-    <t>Powiat nowodworski</t>
-  </si>
-  <si>
-    <t>Powiat ostroĹ‚Ä™cki</t>
-  </si>
-  <si>
-    <t>Powiat ostrowski</t>
-  </si>
-  <si>
-    <t>Powiat otwocki</t>
-  </si>
-  <si>
-    <t>Powiat piaseczyĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat pĹ‚ocki</t>
-  </si>
-  <si>
-    <t>Powiat pĹ‚oĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat pruszkowski</t>
-  </si>
-  <si>
-    <t>Powiat przasnyski</t>
-  </si>
-  <si>
-    <t>Powiat przysuski</t>
-  </si>
-  <si>
-    <t>Powiat puĹ‚tuski</t>
-  </si>
-  <si>
-    <t>Powiat radomski</t>
-  </si>
-  <si>
-    <t>Powiat siedlecki</t>
-  </si>
-  <si>
-    <t>Powiat sierpecki</t>
-  </si>
-  <si>
-    <t>Powiat sochaczewski</t>
-  </si>
-  <si>
-    <t>Powiat sokoĹ‚owski</t>
-  </si>
-  <si>
-    <t>Powiat szydĹ‚owiecki</t>
-  </si>
-  <si>
-    <t>Powiat warszawski zachodni</t>
-  </si>
-  <si>
-    <t>Powiat wÄ™growski</t>
-  </si>
-  <si>
-    <t>Powiat woĹ‚omiĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat wyszkowski</t>
-  </si>
-  <si>
-    <t>Powiat zwoleĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat ĹĽuromiĹ„ski</t>
-  </si>
-  <si>
-    <t>Powiat ĹĽyrardowski</t>
-  </si>
-  <si>
-    <t>Powiat m. OstroĹ‚Ä™ka</t>
-  </si>
-  <si>
-    <t>Powiat m. PĹ‚ock</t>
-  </si>
-  <si>
-    <t>Powiat m. Radom</t>
-  </si>
-  <si>
-    <t>Powiat m. Siedlce</t>
-  </si>
-  <si>
-    <t>Powiat m. st. Warszawa</t>
-  </si>
-  <si>
     <t>exp_per1</t>
   </si>
   <si>
@@ -255,6 +129,132 @@
   </si>
   <si>
     <t>POWIAT</t>
+  </si>
+  <si>
+    <t>powiat białobrzeski</t>
+  </si>
+  <si>
+    <t>powiat ciechanowski</t>
+  </si>
+  <si>
+    <t>powiat garwoliński</t>
+  </si>
+  <si>
+    <t>powiat gostyniński</t>
+  </si>
+  <si>
+    <t>powiat grójecki</t>
+  </si>
+  <si>
+    <t>powiat grodziski</t>
+  </si>
+  <si>
+    <t>powiat kozienicki</t>
+  </si>
+  <si>
+    <t>powiat legionowski</t>
+  </si>
+  <si>
+    <t>powiat lipski</t>
+  </si>
+  <si>
+    <t>powiat makowski</t>
+  </si>
+  <si>
+    <t>powiat nowodworski</t>
+  </si>
+  <si>
+    <t>powiat ostrowski</t>
+  </si>
+  <si>
+    <t>powiat otwocki</t>
+  </si>
+  <si>
+    <t>powiat pruszkowski</t>
+  </si>
+  <si>
+    <t>powiat przasnyski</t>
+  </si>
+  <si>
+    <t>powiat przysuski</t>
+  </si>
+  <si>
+    <t>powiat radomski</t>
+  </si>
+  <si>
+    <t>powiat siedlecki</t>
+  </si>
+  <si>
+    <t>powiat sierpecki</t>
+  </si>
+  <si>
+    <t>powiat sochaczewski</t>
+  </si>
+  <si>
+    <t>powiat warszawski zachodni</t>
+  </si>
+  <si>
+    <t>powiat wyszkowski</t>
+  </si>
+  <si>
+    <t>powiat łosicki</t>
+  </si>
+  <si>
+    <t>powiat miński</t>
+  </si>
+  <si>
+    <t>powiat mławski</t>
+  </si>
+  <si>
+    <t>powiat płocki</t>
+  </si>
+  <si>
+    <t>powiat pułtuski</t>
+  </si>
+  <si>
+    <t>powiat sokołowski</t>
+  </si>
+  <si>
+    <t>powiat szydłowiecki</t>
+  </si>
+  <si>
+    <t>powiat ostrołęcki</t>
+  </si>
+  <si>
+    <t>powiat węgrowski</t>
+  </si>
+  <si>
+    <t>powiat piaseczyński</t>
+  </si>
+  <si>
+    <t>powiat płoński</t>
+  </si>
+  <si>
+    <t>powiat wołomiński</t>
+  </si>
+  <si>
+    <t>powiat zwoleński</t>
+  </si>
+  <si>
+    <t>powiat żuromiński</t>
+  </si>
+  <si>
+    <t>powiat żyrardowski</t>
+  </si>
+  <si>
+    <t>powiat Radom</t>
+  </si>
+  <si>
+    <t>powiat Siedlce</t>
+  </si>
+  <si>
+    <t>powiat Ostrołęka</t>
+  </si>
+  <si>
+    <t>powiat Płock</t>
+  </si>
+  <si>
+    <t>powiat Warszawa</t>
   </si>
 </sst>
 </file>
@@ -676,94 +676,94 @@
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="P2" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="Q2" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="R2" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="S2" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="T2" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="U2" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="V2" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="W2" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="X2" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="Y2" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="Z2" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="AA2" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="AB2" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="AC2" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="AD2" t="s">
-        <v>71</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -886,7 +886,7 @@
         <v>01</v>
       </c>
       <c r="C4" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D4" s="1">
         <v>1006.68</v>
@@ -993,7 +993,7 @@
         <v>02</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1">
         <v>929.16</v>
@@ -1100,7 +1100,7 @@
         <v>03</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="D6" s="1">
         <v>929.12</v>
@@ -1207,7 +1207,7 @@
         <v>04</v>
       </c>
       <c r="C7" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1">
         <v>992.63</v>
@@ -1314,7 +1314,7 @@
         <v>05</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D8" s="1">
         <v>814.44</v>
@@ -1421,7 +1421,7 @@
         <v>06</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1">
         <v>896.62</v>
@@ -1528,7 +1528,7 @@
         <v>07</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1">
         <v>1047.6099999999999</v>
@@ -1635,7 +1635,7 @@
         <v>08</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="D11" s="1">
         <v>734.25</v>
@@ -1742,7 +1742,7 @@
         <v>09</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="D12" s="1">
         <v>1289.51</v>
@@ -1849,7 +1849,7 @@
         <v>10</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="D13" s="1">
         <v>1064.74</v>
@@ -1956,7 +1956,7 @@
         <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D14" s="1">
         <v>983.58</v>
@@ -2063,7 +2063,7 @@
         <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="D15" s="1">
         <v>838.84</v>
@@ -2170,7 +2170,7 @@
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="D16" s="1">
         <v>803.16</v>
@@ -2277,7 +2277,7 @@
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="D17" s="1">
         <v>679.52</v>
@@ -2384,7 +2384,7 @@
         <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="D18" s="1">
         <v>779.76</v>
@@ -2491,7 +2491,7 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D19" s="1">
         <v>822.57</v>
@@ -2598,7 +2598,7 @@
         <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="D20" s="1">
         <v>848.16</v>
@@ -2705,7 +2705,7 @@
         <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D21" s="1">
         <v>990.4</v>
@@ -2812,7 +2812,7 @@
         <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="D22" s="1">
         <v>766.71</v>
@@ -2919,7 +2919,7 @@
         <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="D23" s="1">
         <v>876.78</v>
@@ -3026,7 +3026,7 @@
         <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D24" s="1">
         <v>777.1</v>
@@ -3133,7 +3133,7 @@
         <v>22</v>
       </c>
       <c r="C25" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D25" s="1">
         <v>1225.06</v>
@@ -3240,7 +3240,7 @@
         <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D26" s="1">
         <v>1394.79</v>
@@ -3347,7 +3347,7 @@
         <v>24</v>
       </c>
       <c r="C27" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="D27" s="1">
         <v>1076.68</v>
@@ -3454,7 +3454,7 @@
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="D28" s="1">
         <v>743.63</v>
@@ -3561,7 +3561,7 @@
         <v>26</v>
       </c>
       <c r="C29" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D29" s="1">
         <v>486.79</v>
@@ -3668,7 +3668,7 @@
         <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D30" s="1">
         <v>1019.62</v>
@@ -3775,7 +3775,7 @@
         <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="D31" s="1">
         <v>889.64</v>
@@ -3882,7 +3882,7 @@
         <v>29</v>
       </c>
       <c r="C32" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="D32" s="1">
         <v>1073.1199999999999</v>
@@ -3989,7 +3989,7 @@
         <v>30</v>
       </c>
       <c r="C33" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="D33" s="1">
         <v>844.53</v>
@@ -4096,7 +4096,7 @@
         <v>32</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="D34" s="1">
         <v>1002.97</v>
@@ -4203,7 +4203,7 @@
         <v>33</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="D35" s="1">
         <v>817.27</v>
@@ -4310,7 +4310,7 @@
         <v>34</v>
       </c>
       <c r="C36" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="D36" s="1">
         <v>669.51</v>
@@ -4417,7 +4417,7 @@
         <v>35</v>
       </c>
       <c r="C37" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="D37" s="1">
         <v>1017.92</v>
@@ -4524,7 +4524,7 @@
         <v>36</v>
       </c>
       <c r="C38" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="D38" s="1">
         <v>826.35</v>
@@ -4631,7 +4631,7 @@
         <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="D39" s="1">
         <v>1055.3699999999999</v>
@@ -4738,7 +4738,7 @@
         <v>38</v>
       </c>
       <c r="C40" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="D40" s="1">
         <v>678.63</v>
@@ -4845,7 +4845,7 @@
         <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="D41" s="3">
         <v>0</v>
@@ -4952,7 +4952,7 @@
         <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="D42" s="3">
         <v>0</v>
@@ -5059,7 +5059,7 @@
         <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="D43" s="3">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>64</v>
       </c>
       <c r="C44" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="D44" s="3">
         <v>0</v>
@@ -5273,7 +5273,7 @@
         <v>65</v>
       </c>
       <c r="C45" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="D45" s="3">
         <v>0</v>

</xml_diff>